<commit_message>
Load the real course prices from the fee schedule
Replace the five placeholder courses with the twelve from the supplied
收費標準, which lists only a course and a fee — material fee is therefore 0
throughout, to be filled per course or per quote where one applies. Keep the
source document under 範本/原始檔/ so the figures can be traced.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FmATSSm8rVRDX1JZwo8hRE
</commit_message>
<xml_diff>
--- a/報價單_HTML/範例資料/courses.xlsx
+++ b/報價單_HTML/範例資料/courses.xlsx
@@ -35,14 +35,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">課輔班</t>
+          <t xml:space="preserve">全科班</t>
         </is>
       </c>
       <c r="B2">
         <v>6000</v>
       </c>
       <c r="C2">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -53,32 +53,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">美語班</t>
+          <t xml:space="preserve">小學美語班</t>
         </is>
       </c>
       <c r="B3">
-        <v>3000</v>
+        <v>3600</v>
       </c>
       <c r="C3">
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">英文班每月計8堂課</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">數學班</t>
+          <t xml:space="preserve">全科美語班</t>
         </is>
       </c>
       <c r="B4">
-        <v>4000</v>
+        <v>9000</v>
       </c>
       <c r="C4">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -89,14 +89,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">作文班</t>
+          <t xml:space="preserve">國中英文班</t>
         </is>
       </c>
       <c r="B5">
-        <v>2800</v>
+        <v>3600</v>
       </c>
       <c r="C5">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -107,16 +107,142 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">理化班</t>
+          <t xml:space="preserve">國中數學班</t>
         </is>
       </c>
       <c r="B6">
-        <v>4500</v>
+        <v>3600</v>
       </c>
       <c r="C6">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">國中生物班</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>3600</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">國中理化班</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>3600</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">國中全科班</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>9000</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">國(高)中家教班</t>
+        </is>
+      </c>
+      <c r="B10">
+        <v>4000</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">高中數學班</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>3600</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">高中英文班</t>
+        </is>
+      </c>
+      <c r="B12">
+        <v>3600</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">英檢班</t>
+        </is>
+      </c>
+      <c r="B13">
+        <v>3600</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>

</xml_diff>